<commit_message>
Extended the list of stocks analyzed; change data preprocessing to both backward and forward fill NAs; added filling the wrongly parsed external ratings with 0s
</commit_message>
<xml_diff>
--- a/output/stock_quant_scores/AAPL_balance_df.xlsx
+++ b/output/stock_quant_scores/AAPL_balance_df.xlsx
@@ -1594,10 +1594,14 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>136522000000</v>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v>9355000000</v>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
         <v>9842000000</v>
@@ -1605,13 +1609,19 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="n">
+        <v>63090000000</v>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>5562000000</v>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="n">
+        <v>287912000000</v>
+      </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
@@ -1620,7 +1630,9 @@
         <v>8382000000</v>
       </c>
       <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
+      <c r="AB6" t="n">
+        <v>125481000000</v>
+      </c>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
@@ -1636,7 +1648,9 @@
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
+      <c r="AP6" t="n">
+        <v>351002000000</v>
+      </c>
       <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
@@ -1657,15 +1671,21 @@
       <c r="BD6" t="inlineStr"/>
       <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="inlineStr"/>
-      <c r="BG6" t="inlineStr"/>
+      <c r="BG6" t="n">
+        <v>134836000000</v>
+      </c>
       <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="inlineStr"/>
+      <c r="BI6" t="n">
+        <v>6580000000</v>
+      </c>
       <c r="BJ6" t="inlineStr"/>
       <c r="BK6" t="inlineStr"/>
       <c r="BL6" t="inlineStr"/>
       <c r="BM6" t="inlineStr"/>
       <c r="BN6" t="inlineStr"/>
-      <c r="BO6" t="inlineStr"/>
+      <c r="BO6" t="n">
+        <v>34940000000</v>
+      </c>
       <c r="BP6" t="inlineStr"/>
       <c r="BQ6" t="inlineStr"/>
     </row>

</xml_diff>